<commit_message>
patch - schedule command, UI cleanup, announce auto-ping team
</commit_message>
<xml_diff>
--- a/data/schedules.xlsx
+++ b/data/schedules.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
   <si>
     <t>ID</t>
   </si>
@@ -43,13 +43,28 @@
     <t>27-05-26</t>
   </si>
   <si>
-    <t>19:00</t>
+    <t>16:30</t>
+  </si>
+  <si>
+    <t>Randoms</t>
+  </si>
+  <si>
+    <t>This is a test</t>
+  </si>
+  <si>
+    <t>Scheduled</t>
+  </si>
+  <si>
+    <t>28-05-26</t>
+  </si>
+  <si>
+    <t>16:00</t>
   </si>
   <si>
     <t>N/A</t>
   </si>
   <si>
-    <t>Scheduled</t>
+    <t>Practice with the tryouts</t>
   </si>
   <si>
     <t>Discord Tag</t>
@@ -107,6 +122,12 @@
   </si>
   <si>
     <t>Added At</t>
+  </si>
+  <si>
+    <t>Sick</t>
+  </si>
+  <si>
+    <t>2026-05-27T14:54:22.793Z</t>
   </si>
   <si>
     <t>Label</t>
@@ -495,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -523,7 +544,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1779837526376</v>
+        <v>1779894380065</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -538,10 +559,33 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1779896831797</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -557,13 +601,13 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
@@ -571,61 +615,61 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
         <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -636,24 +680,41 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -669,18 +730,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>